<commit_message>
Q425 Earnings Season pt.2
</commit_message>
<xml_diff>
--- a/Financial Analysis/ADBE.xlsx
+++ b/Financial Analysis/ADBE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\antos\Documents\GitHub\FinanceModels\Financial Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E347E133-1BF4-49D6-B1FE-C2D7C89CD371}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C5F4F72-6C65-428C-8C4B-D8C5AA4D6B46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{030F5AE8-2ADC-4446-9A99-98294E370635}"/>
   </bookViews>
@@ -848,14 +848,14 @@
         <v>1</v>
       </c>
       <c r="D3" s="6">
-        <v>271.73</v>
+        <v>261.24</v>
       </c>
       <c r="E3" s="4">
-        <v>46059</v>
+        <v>46070</v>
       </c>
       <c r="F3" s="4">
         <f ca="1">TODAY()</f>
-        <v>46059</v>
+        <v>46070</v>
       </c>
       <c r="G3" s="4">
         <v>46093</v>
@@ -889,7 +889,7 @@
       </c>
       <c r="D5" s="5">
         <f>D3*D4</f>
-        <v>113311.41</v>
+        <v>108937.08</v>
       </c>
       <c r="I5" s="11" t="s">
         <v>39</v>
@@ -942,7 +942,7 @@
       </c>
       <c r="D9" s="5">
         <f>D5-D8</f>
-        <v>113764.41</v>
+        <v>109390.08</v>
       </c>
     </row>
   </sheetData>
@@ -7436,7 +7436,7 @@
       </c>
       <c r="BD38" s="6">
         <f>Main!D3</f>
-        <v>271.73</v>
+        <v>261.24</v>
       </c>
     </row>
     <row r="39" spans="2:56" x14ac:dyDescent="0.3">
@@ -7445,7 +7445,7 @@
       </c>
       <c r="BD39" s="13">
         <f>BD37/BD38-1</f>
-        <v>0.33696027720687871</v>
+        <v>0.39064544528182954</v>
       </c>
     </row>
     <row r="40" spans="2:56" x14ac:dyDescent="0.3">

</xml_diff>